<commit_message>
Reset stats on keyboard disconnect, publication prep, user manual
Disconnecting the tracked keyboard now stops the metronome and clears
stats/graph/message, matching a fresh launch (RhythmEngine.onSourceLost).
Cahier des charges renamed to JustRhythm (v2.1), EX-003 updated for the
English/French localization, Paramètres and Risques sections brought up to
date with the sync merge and reward feature. Publication guide expanded with
the TestFlight tester setup, full submission walkthrough, and encryption
compliance steps. Adds a full English user manual (Tutorial/user-manual.md).
</commit_message>
<xml_diff>
--- a/JustRhythm/cahier-des-charges-just-rhythm-natif.xlsx
+++ b/JustRhythm/cahier-des-charges-just-rhythm-natif.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="880" windowWidth="16380" windowHeight="8200" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="860" windowWidth="36000" windowHeight="22520" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Contexte" sheetId="1" state="visible" r:id="rId1"/>
@@ -240,7 +240,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -332,9 +332,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -594,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -604,14 +612,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cahier des charges — « Fil à plomb », version native</t>
+          <t>Cahier des charges — « JustRhythm », version native</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Application iPhone d'entraînement à la précision rythmique au piano · v2.0 · rédigé par Raphaël</t>
+          <t>Application iPhone d'entraînement à la précision rythmique au piano · v2.1 · rédigé par Raphaël</t>
         </is>
       </c>
     </row>
@@ -804,89 +812,97 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="51.75" customHeight="1">
+    <row r="42" ht="68" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
+          <t>v2.1 — Localisation anglais/français, retour de justesse, fusion synchro. Base anglaise avec traduction française automatique selon la langue de l'iPhone (catalogue de chaînes Localizable.xcstrings) ; notation des notes adaptée à la langue (lettres C/D/E… ou solfège Do/Ré/Mi selon le cas). Ajout d'un retour de justesse optionnel sur l'instrument, en deux modes : note doublée à l'octave ou note muette si imprécise (EX-130 / EX-131). Fusion du suivi d'horloge MIDI dans le réglage de démarrage synchronisé (EX-053 / EX-054) : plus de bascule séparée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="51.75" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
           <t>v2.0 — Version native. Refonte complète de l'interface en vocabulaire système ; nouveau bloc d'exigences « Style et plateforme » (EX-110 à EX-118) ; séparation des réglages d'usage et de configuration (EX-096) ; ajout d'un bloc « Publication » (EX-120 à EX-124). Périmètre resserré à 40 exigences en phase 1. Deux fonctions retirées après essai : retour haptique et portrait inversé.</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>v1.0 à v1.3 — Versions antérieures, interface à identité graphique propre. Conservées pour mémoire, plus maintenues.</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+    <row r="45" ht="30" customHeight="1"/>
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>Synthèse (calculée depuis l'onglet Exigences)</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>Phase 1 — Indispensable</t>
         </is>
       </c>
-      <c r="B46" s="6">
+      <c r="B47" s="6">
         <f>COUNTIFS(Exigences!$E$3:$E$200,"Indispensable",Exigences!$G$3:$G$200,"1")</f>
         <v/>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>Phase 1 — Important</t>
         </is>
       </c>
-      <c r="B47" s="6">
+      <c r="B48" s="6">
         <f>COUNTIFS(Exigences!$E$3:$E$200,"Important",Exigences!$G$3:$G$200,"1")</f>
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>Phase 1 — Souhaitable</t>
         </is>
       </c>
-      <c r="B48" s="6">
+      <c r="B49" s="6">
         <f>COUNTIFS(Exigences!$E$3:$E$200,"Souhaitable",Exigences!$G$3:$G$200,"1")</f>
         <v/>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>Phase 1 — total</t>
         </is>
       </c>
-      <c r="B49" s="6">
+      <c r="B50" s="6">
         <f>COUNTIF(Exigences!$G$3:$G$200,"1")</f>
         <v/>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>Phase 2 — reporté</t>
         </is>
       </c>
-      <c r="B50" s="6">
+      <c r="B51" s="6">
         <f>COUNTIF(Exigences!$G$3:$G$200,"2")</f>
         <v/>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>Total décrit</t>
         </is>
       </c>
-      <c r="B51" s="6">
+      <c r="B52" s="6">
         <f>COUNTA(Exigences!$A$3:$A$200)</f>
         <v/>
       </c>
@@ -912,7 +928,7 @@
     <col width="201.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" style="39" min="7" max="7"/>
     <col width="58.6640625" bestFit="1" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -947,7 +963,7 @@
           <t>Réglage / valeur</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="37" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
@@ -1089,12 +1105,12 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>L'interface est en français.</t>
+          <t>L'application s'affiche dans la langue réglée sur mon iPhone, sans réglage à faire dans l'app.</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Libellés en français, écarts en millisecondes, notes nommées Do / Ré / Mi.</t>
+          <t>Anglais par défaut (langue source), français traduit automatiquement quand l'iPhone est en français ; écarts en millisecondes, identiques dans les deux langues ; notes nommées en lettres (C, D, E…) sauf en français, où elles restent en solfège (Do, Ré, Mi).</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -1104,7 +1120,7 @@
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>fr-FR</t>
+          <t>suit iOS</t>
         </is>
       </c>
       <c r="G5" s="13" t="inlineStr">
@@ -1112,7 +1128,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="H5" s="14" t="n"/>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>catalogue de chaînes (Localizable.xcstrings), testé en simulateur le 28/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="27.75" customHeight="1">
       <c r="A6" s="15" t="inlineStr">
@@ -1791,8 +1811,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G23" s="18" t="n">
-        <v>3</v>
+      <c r="G23" s="18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="H23" s="14" t="n"/>
     </row>
@@ -2769,12 +2791,12 @@
           <t>désactivé</t>
         </is>
       </c>
-      <c r="G49" s="35" t="inlineStr">
+      <c r="G49" s="38" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="H49" s="36" t="inlineStr">
+      <c r="H49" s="35" t="inlineStr">
         <is>
           <t>sert surtout à régler l'alignement à l'oreille contre une référence matérielle</t>
         </is>
@@ -2801,7 +2823,7 @@
           <t>Suivi de l'horloge MIDI (24 impulsions par noire). Période lissée et phase corrigée par un décalage d'ancrage borné, sans rupture de grille. Le tempo reçu est affiché à la place du tempo réglé, qui ne fait plus foi. S'active et se désactive avec EX-053 : un seul réglage « Démarrage synchronisé » commande les deux, il n'y a jamais de cas où l'un est utile sans l'autre.</t>
         </is>
       </c>
-      <c r="E50" s="37" t="inlineStr">
+      <c r="E50" s="36" t="inlineStr">
         <is>
           <t>Souhaitable</t>
         </is>
@@ -2811,12 +2833,12 @@
           <t>suit EX-053</t>
         </is>
       </c>
-      <c r="G50" s="35" t="inlineStr">
+      <c r="G50" s="38" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="H50" s="36" t="inlineStr">
+      <c r="H50" s="35" t="inlineStr">
         <is>
           <t>sans lui, Start donne le départ mais pas le tempo : la dérive est inévitable — fusionné avec EX-053 le 27/07/2026, l'usage a confirmé qu'ils ne se séparent jamais</t>
         </is>
@@ -4081,7 +4103,7 @@
           <t>Un réglage « Récompense sonore » dans les Réglages, désactivé par défaut. Actif, il déclenche un message MIDI vers l'instrument à chaque frappe tombée dans la zone « juste », coupé par un Note Off peu après pour ne jamais laisser de note tenue.</t>
         </is>
       </c>
-      <c r="E84" s="37" t="inlineStr">
+      <c r="E84" s="36" t="inlineStr">
         <is>
           <t>Souhaitable</t>
         </is>
@@ -4091,12 +4113,12 @@
           <t>désactivé</t>
         </is>
       </c>
-      <c r="G84" s="35" t="inlineStr">
+      <c r="G84" s="38" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="H84" s="36" t="inlineStr">
+      <c r="H84" s="35" t="inlineStr">
         <is>
           <t>testé et validé sur mon clavier le 27/07/2026</t>
         </is>
@@ -4123,7 +4145,7 @@
           <t>Un sélecteur à deux choix dans les Réglages, actif seulement si EX-130 l'est. « Note doublée à l'octave » : la frappe juste ajoute une note un octave au-dessus. « Note muette si imprécise » : seule une frappe juste est renvoyée par l'application, à la même hauteur ; une frappe imprécise reste silencieuse.</t>
         </is>
       </c>
-      <c r="E85" s="37" t="inlineStr">
+      <c r="E85" s="36" t="inlineStr">
         <is>
           <t>Souhaitable</t>
         </is>
@@ -4133,12 +4155,12 @@
           <t>note à l'octave</t>
         </is>
       </c>
-      <c r="G85" s="35" t="inlineStr">
+      <c r="G85" s="38" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="H85" s="36" t="inlineStr">
+      <c r="H85" s="35" t="inlineStr">
         <is>
           <t>le mode muet suppose le Local Control coupé sur l'instrument, sinon il joue déjà tout seul en local</t>
         </is>
@@ -4157,7 +4179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4623,37 +4645,117 @@
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
+          <t>suit EX-053</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>réglages (via Démarrage synchronisé)</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>EX-054</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>exige que le clavier émette du MIDI Clock ; certains n'envoient que Start et Stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="27.75" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Récompense sonore</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
           <t>désactivé</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E12" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F12" s="16" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
         <is>
           <t>réglages</t>
         </is>
       </c>
-      <c r="G12" s="15" t="inlineStr">
-        <is>
-          <t>EX-054</t>
-        </is>
-      </c>
-      <c r="H12" s="14" t="inlineStr">
-        <is>
-          <t>exige que le clavier émette du MIDI Clock ; certains n'envoient que Start et Stop</t>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>EX-130</t>
+        </is>
+      </c>
+      <c r="H13" s="14" t="n"/>
+    </row>
+    <row r="14" ht="27.75" customHeight="1">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Mode de récompense</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>note à l'octave</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>réglages</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>EX-131</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>deux options : note à l'octave, ou note muette si imprécise</t>
         </is>
       </c>
     </row>
@@ -4669,7 +4771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5079,6 +5181,29 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="45.75" customHeight="1">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>Suivi d'horloge séparé du démarrage synchronisé</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>Les deux réglages étaient indépendants, mais jamais utilisés l'un sans l'autre en pratique : sans le démarrage synchronisé, le suivi d'horloge n'a pas de sens.</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>Fusionnés en un seul réglage « Démarrage synchronisé » (EX-053), qui active aussi le suivi d'horloge (EX-054). Plus de bascule séparée dans les Réglages.</t>
+        </is>
+      </c>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>Un réglage inutile dans l'interface, qui complique le choix sans offrir de cas d'usage réel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="45.75" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Fix MIDI clock sync drift, disable Start while waiting, multi-channel input
Two real bugs in the clock-following sync (EX-053/054): a data race on the
grid state (anchor/period/stepIndex/nextStep) between the scheduler queue and
the main-thread note handler, and a stepIndex-multiplied noise amplification
in the phase correction that turned tiny period-estimate jitter into a
growing drift over tens of seconds. Both fixed — confirmed on hardware, down
to ~2ms of normal MIDI jitter. The Start button now disables while synced
start is waiting for the keyboard's trigger, Stop stays available once
running. MIDI channel filtering moves from a single channel to a multi-select
(EX-017), with a dedicated Settings screen (ChannelSelectionView).
</commit_message>
<xml_diff>
--- a/JustRhythm/cahier-des-charges-just-rhythm-natif.xlsx
+++ b/JustRhythm/cahier-des-charges-just-rhythm-natif.xlsx
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -619,7 +619,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Application iPhone d'entraînement à la précision rythmique au piano · v2.1 · rédigé par Raphaël</t>
+          <t>Application iPhone d'entraînement à la précision rythmique au piano · v2.2 · rédigé par Raphaël</t>
         </is>
       </c>
     </row>
@@ -812,97 +812,104 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="68" customHeight="1">
+    <row r="42" ht="82" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
+          <t>v2.2 — Fiabilité du suivi d'horloge, canaux MIDI multiples. Corrige deux bugs de la synchronisation sur l'horloge du clavier (EX-053 / EX-054) : une course sans verrou sur l'état de la grille, et une amplification du bruit de mesure par stepIndex qui faisait dériver la synchro de quelques ms à un décalage important en quelques dizaines de secondes. Le bouton Start se désactive tant que la synchro attend son déclenchement par le clavier. L'écoute MIDI accepte maintenant plusieurs canaux à la fois, pas un seul (EX-017).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="68" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
           <t>v2.1 — Localisation anglais/français, retour de justesse, fusion synchro. Base anglaise avec traduction française automatique selon la langue de l'iPhone (catalogue de chaînes Localizable.xcstrings) ; notation des notes adaptée à la langue (lettres C/D/E… ou solfège Do/Ré/Mi selon le cas). Ajout d'un retour de justesse optionnel sur l'instrument, en deux modes : note doublée à l'octave ou note muette si imprécise (EX-130 / EX-131). Fusion du suivi d'horloge MIDI dans le réglage de démarrage synchronisé (EX-053 / EX-054) : plus de bascule séparée.</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="51.75" customHeight="1">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="44" ht="51.75" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>v2.0 — Version native. Refonte complète de l'interface en vocabulaire système ; nouveau bloc d'exigences « Style et plateforme » (EX-110 à EX-118) ; séparation des réglages d'usage et de configuration (EX-096) ; ajout d'un bloc « Publication » (EX-120 à EX-124). Périmètre resserré à 40 exigences en phase 1. Deux fonctions retirées après essai : retour haptique et portrait inversé.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>v1.0 à v1.3 — Versions antérieures, interface à identité graphique propre. Conservées pour mémoire, plus maintenues.</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="30" customHeight="1"/>
-    <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="3" t="inlineStr">
+    <row r="46" ht="16" customHeight="1"/>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>Synthèse (calculée depuis l'onglet Exigences)</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>Phase 1 — Indispensable</t>
         </is>
       </c>
-      <c r="B47" s="6">
+      <c r="B48" s="6">
         <f>COUNTIFS(Exigences!$E$3:$E$200,"Indispensable",Exigences!$G$3:$G$200,"1")</f>
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>Phase 1 — Important</t>
         </is>
       </c>
-      <c r="B48" s="6">
+      <c r="B49" s="6">
         <f>COUNTIFS(Exigences!$E$3:$E$200,"Important",Exigences!$G$3:$G$200,"1")</f>
         <v/>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>Phase 1 — Souhaitable</t>
         </is>
       </c>
-      <c r="B49" s="6">
+      <c r="B50" s="6">
         <f>COUNTIFS(Exigences!$E$3:$E$200,"Souhaitable",Exigences!$G$3:$G$200,"1")</f>
         <v/>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>Phase 1 — total</t>
         </is>
       </c>
-      <c r="B50" s="6">
+      <c r="B51" s="6">
         <f>COUNTIF(Exigences!$G$3:$G$200,"1")</f>
         <v/>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>Phase 2 — reporté</t>
         </is>
       </c>
-      <c r="B51" s="6">
+      <c r="B52" s="6">
         <f>COUNTIF(Exigences!$G$3:$G$200,"2")</f>
         <v/>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>Total décrit</t>
         </is>
       </c>
-      <c r="B52" s="6">
+      <c r="B53" s="6">
         <f>COUNTA(Exigences!$A$3:$A$200)</f>
         <v/>
       </c>
@@ -1943,12 +1950,12 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Je peux restreindre la mesure à un canal MIDI.</t>
+          <t>Je peux restreindre la mesure à un ou plusieurs canaux MIDI.</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Choix « tous » ou 1 à 16.</t>
+          <t>Choix « tous les canaux » ou sélection multiple parmi 1 à 16 (ex. clavier multitimbral réparti sur plusieurs canaux : 1, 9, 10).</t>
         </is>
       </c>
       <c r="E27" s="19" t="inlineStr">
@@ -1966,7 +1973,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="H27" s="14" t="n"/>
+      <c r="H27" s="14" t="inlineStr">
+        <is>
+          <t>passé de canal unique à sélection multiple (Set&lt;Int&gt;), écran dédié dans Réglages</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="27.75" customHeight="1">
       <c r="A28" s="15" t="inlineStr">
@@ -4771,7 +4782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5203,7 +5214,50 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="45.75" customHeight="1"/>
+    <row r="21" ht="45.75" customHeight="1">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>Course sur l'état de la grille</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>anchor/period/stepIndex/nextStep étaient écrits depuis la queue de scheduling (schedule, followClock) et lus depuis la queue principale (nearestStep, à chaque note jouée) sans aucune synchronisation.</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>Un verrou (NSLock) protège désormais les quatre variables, en lecture comme en écriture, quelle que soit la queue d'où l'accès a lieu.</t>
+        </is>
+      </c>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>Un écart de justesse incohérent et différent à chaque fois, uniquement quand la synchro d'horloge est active — très difficile à diagnostiquer sans relire tout le threading.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45.75" customHeight="1">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>Amplification du bruit par stepIndex dans le suivi d'horloge</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>Recalculer nextStep = anchor + stepIndex * newPeriod à chaque correction multipliait le moindre bruit de mesure de période par stepIndex, qui ne fait que grandir pendant la séance : quelques dixièmes de ms de bruit devenaient un saut de plusieurs dizaines de ms après quelques dizaines de secondes.</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>Réancrage local à chaque correction de phase, stepIndex remis à 0 à chaque fois : l'erreur reste bornée par la correction de phase (±20 ms), elle ne peut plus être amplifiée par la durée de la séance.</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>La synchro sur l'horloge du clavier devient inutilisable au bout de quelques dizaines de secondes, un symptôme qui grandit avec la durée — facile à confondre avec un simple problème de gigue matérielle.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Grid-relative accuracy, tuner readout, keyboard tempo adoption
Zone and scale become relative to the subdivision: the "right" zone is a
percentage of the grid step with a 20 ms floor, and the graph is capped at
half a subdivision — the range an error can actually reach. Same shape as the
existing Regularity threshold, for the same reason: a percentage alone would
eventually demand more precision than a hand can deliver.

Replaces the last-note readout, too jumpy to steer by, with a tuner-style
one over the last 16 notes (BiasMeter). It reads the range those notes land
in, not just their average — early and late errors cancel out in a mean, so
an average alone called scattered playing perfect. Both triangles light for
that case, hence the new "uneven" verdict.

The tempo received over MIDI clock is now adopted as the app's own and kept
after stopping, with the tempo controls disabled while the clock drives.
</commit_message>
<xml_diff>
--- a/JustRhythm/cahier-des-charges-just-rhythm-natif.xlsx
+++ b/JustRhythm/cahier-des-charges-just-rhythm-natif.xlsx
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -619,7 +619,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Application iPhone d'entraînement à la précision rythmique au piano · v2.2 · rédigé par Raphaël</t>
+          <t>Application iPhone d'entraînement à la précision rythmique au piano · v2.4 · rédigé par Raphaël</t>
         </is>
       </c>
     </row>
@@ -815,101 +815,114 @@
     <row r="42" ht="82" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
+          <t>v2.4 — Lecture instantanée sur la fourchette glissante. L'écart de la dernière note, trop instable pour qu'on s'y fie en jouant, cède la place à trois voyants façon accordeur, alimentés par la moyenne et la dispersion des 16 dernières notes (EX-066 / EX-089, cette dernière passant en phase 1) : les deux côtés s'allument séparément, ce qui distingue un décalage systématique d'un jeu irrégulier. Le tempo reçu du clavier est désormais adopté par l'application et conservé après l'arrêt, les commandes de tempo étant neutralisées tant que l'horloge pilote (EX-054).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="82" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>v2.3 — Zone juste et échelle rapportées à la subdivision. La zone « juste » s'exprime en pourcentage de la subdivision plutôt qu'en millisecondes absolues, avec un plancher à 20 ms (EX-063) : elle se resserre d'elle-même quand la grille s'affine, sans jamais exiger mieux que le seuil de perception. L'échelle du graphe est bornée à la demi-subdivision, seule plage qu'un écart puisse atteindre, le curseur ne servant plus qu'à resserrer (EX-067). Les deux suivent l'horloge du clavier quand elle est suivie, et non le tempo réglé à la main.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="82" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
           <t>v2.2 — Fiabilité du suivi d'horloge, canaux MIDI multiples. Corrige deux bugs de la synchronisation sur l'horloge du clavier (EX-053 / EX-054) : une course sans verrou sur l'état de la grille, et une amplification du bruit de mesure par stepIndex qui faisait dériver la synchro de quelques ms à un décalage important en quelques dizaines de secondes. Le bouton Start se désactive tant que la synchro attend son déclenchement par le clavier. L'écoute MIDI accepte maintenant plusieurs canaux à la fois, pas un seul (EX-017).</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="68" customHeight="1">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="45" ht="68" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>v2.1 — Localisation anglais/français, retour de justesse, fusion synchro. Base anglaise avec traduction française automatique selon la langue de l'iPhone (catalogue de chaînes Localizable.xcstrings) ; notation des notes adaptée à la langue (lettres C/D/E… ou solfège Do/Ré/Mi selon le cas). Ajout d'un retour de justesse optionnel sur l'instrument, en deux modes : note doublée à l'octave ou note muette si imprécise (EX-130 / EX-131). Fusion du suivi d'horloge MIDI dans le réglage de démarrage synchronisé (EX-053 / EX-054) : plus de bascule séparée.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="51.75" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="46" ht="51.75" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>v2.0 — Version native. Refonte complète de l'interface en vocabulaire système ; nouveau bloc d'exigences « Style et plateforme » (EX-110 à EX-118) ; séparation des réglages d'usage et de configuration (EX-096) ; ajout d'un bloc « Publication » (EX-120 à EX-124). Périmètre resserré à 40 exigences en phase 1. Deux fonctions retirées après essai : retour haptique et portrait inversé.</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>v1.0 à v1.3 — Versions antérieures, interface à identité graphique propre. Conservées pour mémoire, plus maintenues.</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="16" customHeight="1"/>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>Synthèse (calculée depuis l'onglet Exigences)</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>Phase 1 — Indispensable</t>
         </is>
       </c>
-      <c r="B48" s="6">
+      <c r="B50" s="6">
         <f>COUNTIFS(Exigences!$E$3:$E$200,"Indispensable",Exigences!$G$3:$G$200,"1")</f>
         <v/>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>Phase 1 — Important</t>
         </is>
       </c>
-      <c r="B49" s="6">
+      <c r="B51" s="6">
         <f>COUNTIFS(Exigences!$E$3:$E$200,"Important",Exigences!$G$3:$G$200,"1")</f>
         <v/>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>Phase 1 — Souhaitable</t>
         </is>
       </c>
-      <c r="B50" s="6">
+      <c r="B52" s="6">
         <f>COUNTIFS(Exigences!$E$3:$E$200,"Souhaitable",Exigences!$G$3:$G$200,"1")</f>
         <v/>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>Phase 1 — total</t>
         </is>
       </c>
-      <c r="B51" s="6">
+      <c r="B53" s="6">
         <f>COUNTIF(Exigences!$G$3:$G$200,"1")</f>
         <v/>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>Phase 2 — reporté</t>
         </is>
       </c>
-      <c r="B52" s="6">
+      <c r="B54" s="6">
         <f>COUNTIF(Exigences!$G$3:$G$200,"2")</f>
         <v/>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>Total décrit</t>
         </is>
       </c>
-      <c r="B53" s="6">
+      <c r="B55" s="6">
         <f>COUNTA(Exigences!$A$3:$A$200)</f>
         <v/>
       </c>
@@ -2831,7 +2844,7 @@
       </c>
       <c r="D50" s="33" t="inlineStr">
         <is>
-          <t>Suivi de l'horloge MIDI (24 impulsions par noire). Période lissée et phase corrigée par un décalage d'ancrage borné, sans rupture de grille. Le tempo reçu est affiché à la place du tempo réglé, qui ne fait plus foi. S'active et se désactive avec EX-053 : un seul réglage « Démarrage synchronisé » commande les deux, il n'y a jamais de cas où l'un est utile sans l'autre.</t>
+          <t>Suivi de l'horloge MIDI (24 impulsions par noire). Période lissée et phase corrigée par un décalage d'ancrage borné, sans rupture de grille. Le tempo reçu est affiché à la place du tempo réglé, qui ne fait plus foi, et il est adopté comme tempo de l'application : les réglages qui en dépendent le suivent, et la valeur survit à l'arrêt de la séance. Les commandes de tempo sont neutralisées tant que l'horloge pilote. S'active et se désactive avec EX-053 : un seul réglage « Démarrage synchronisé » commande les deux, il n'y a jamais de cas où l'un est utile sans l'autre.</t>
         </is>
       </c>
       <c r="E50" s="36" t="inlineStr">
@@ -2851,7 +2864,7 @@
       </c>
       <c r="H50" s="35" t="inlineStr">
         <is>
-          <t>sans lui, Start donne le départ mais pas le tempo : la dérive est inévitable — fusionné avec EX-053 le 27/07/2026, l'usage a confirmé qu'ils ne se séparent jamais</t>
+          <t>sans lui, Start donne le départ mais pas le tempo : la dérive est inévitable — fusionné avec EX-053 le 27/07/2026, l'usage a confirmé qu'ils ne se séparent jamais ; tempo reçu rendu persistant le 29/07/2026</t>
         </is>
       </c>
     </row>
@@ -2982,12 +2995,12 @@
       </c>
       <c r="C54" s="16" t="inlineStr">
         <is>
-          <t>Une bande matérialise la zone que je considère comme « dans le temps ».</t>
+          <t>Une bande matérialise la zone que je considère comme « dans le temps », et sa largeur tient compte de la finesse de la grille.</t>
         </is>
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>Largeur réglable, visible en permanence de part et d'autre de la ligne.</t>
+          <t>Largeur réglable en pourcentage de la subdivision, visible en permanence de part et d'autre de la ligne. Seuil au plus permissif entre le pourcentage réglé et 20 ms : en deçà l'écart cesse de s'entendre, l'exiger n'aurait pas de sens. Même forme que le seuil de régularité (EX-082).</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -2997,7 +3010,7 @@
       </c>
       <c r="F54" s="16" t="inlineStr">
         <is>
-          <t>± 20 ms</t>
+          <t>5 % ou 20 ms</t>
         </is>
       </c>
       <c r="G54" s="13" t="inlineStr">
@@ -3005,7 +3018,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="H54" s="14" t="n"/>
+      <c r="H54" s="14" t="inlineStr">
+        <is>
+          <t>passée d'une largeur absolue en ms à un pourcentage de la subdivision : ±50 ms valent 5 % d'une noire à 60 bpm mais 43 % d'une double-croche à 128 bpm</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="27.75" customHeight="1">
       <c r="A55" s="10" t="inlineStr">
@@ -3020,12 +3037,12 @@
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>Un affichage instantané en gros caractères donne l'écart de la dernière note.</t>
+          <t>Une lecture instantanée me dit où j'en suis sans que j'aie à quitter le clavier des yeux.</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>Valeur en millisecondes plus un mot. Lisible à un mètre depuis le pupitre.</t>
+          <t>Trois voyants, façon accordeur : un triangle de chaque côté et une barre centrale. La barre ne s'allume que si la fourchette des dernières notes (EX-089) tient entière dans la zone juste ; sinon un triangle s'allume du côté du débordement, et les deux ensemble quand le jeu est irrégulier. Sous les voyants, un mot — dans le temps, en avance, en retard, irrégulier — et la fourchette chiffrée en petit, seule à porter l'ampleur du décalage. Jamais la dernière note. Lisible à un mètre depuis le pupitre.</t>
         </is>
       </c>
       <c r="E55" s="12" t="inlineStr">
@@ -3043,7 +3060,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="H55" s="14" t="n"/>
+      <c r="H55" s="14" t="inlineStr">
+        <is>
+          <t>l'écart de la dernière note sautait d'une frappe à l'autre : impossible de s'en servir pour se corriger en jouant — remplacé le 29/07/2026, d'abord par neuf barres graduées, réduites à trois voyants après essai (voir Risques et décisions)</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="34.5" customHeight="1">
       <c r="A56" s="15" t="inlineStr">
@@ -3208,12 +3229,12 @@
       </c>
       <c r="C60" s="16" t="inlineStr">
         <is>
-          <t>Je règle l'échelle horizontale selon mon niveau du jour.</t>
+          <t>Je règle l'échelle horizontale selon mon niveau du jour, sans qu'elle puisse mentir sur la plage réellement atteignable.</t>
         </is>
       </c>
       <c r="D60" s="16" t="inlineStr">
         <is>
-          <t>De ±40 ms à ±300 ms.</t>
+          <t>Bornée à la demi-subdivision, plage qu'un écart ne peut par construction jamais dépasser (EX-032). Curseur de resserrement de 25 % à 100 % de cette plage.</t>
         </is>
       </c>
       <c r="E60" s="19" t="inlineStr">
@@ -3223,15 +3244,19 @@
       </c>
       <c r="F60" s="16" t="inlineStr">
         <is>
-          <t>± 120 ms</t>
+          <t>100 % (½ subdivision)</t>
         </is>
       </c>
       <c r="G60" s="18" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H60" s="14" t="n"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H60" s="14" t="inlineStr">
+        <is>
+          <t>au-delà de la demi-subdivision le graphe montrait du vide, en deçà il écrasait les notes contre le bord</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="27.75" customHeight="1">
       <c r="A61" s="10" t="inlineStr">
@@ -3515,7 +3540,7 @@
       </c>
       <c r="D68" s="16" t="inlineStr">
         <is>
-          <t>Moyenne glissante des X dernières notes, X réglable de 4 à 32.</t>
+          <t>Moyenne et dispersion des 16 dernières notes, les deux ensemble. Elles alimentent la lecture instantanée (EX-066). La moyenne seule ne suffit pas : les avances y annulent les retards, si bien qu'un jeu dispersé mais centré afficherait le même chiffre qu'un jeu propre. Fenêtre fixe pour l'instant, la rendre réglable reste ouvert.</t>
         </is>
       </c>
       <c r="E68" s="17" t="inlineStr">
@@ -3528,10 +3553,16 @@
           <t>8 notes</t>
         </is>
       </c>
-      <c r="G68" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="H68" s="14" t="n"/>
+      <c r="G68" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H68" s="14" t="inlineStr">
+        <is>
+          <t>16 notes : assez pour noyer la variabilité d'une frappe isolée, assez peu pour qu'une correction du jeu se voie en une ou deux mesures</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="27.75" customHeight="1">
       <c r="A69" s="10" t="inlineStr">
@@ -4280,7 +4311,11 @@
           <t>EX-040</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>recopié depuis l'horloge du clavier quand elle est suivie, et conservé après l'arrêt</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="27.75" customHeight="1">
       <c r="A3" s="11" t="inlineStr">
@@ -4408,22 +4443,22 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>± 20</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>± 5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>± 60</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>ms</t>
+          <t>% de la subdivision</t>
         </is>
       </c>
       <c r="F6" s="16" t="inlineStr">
@@ -4438,7 +4473,7 @@
       </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
-          <t>20 ms est le seuil courant de perception d'un décalage</t>
+          <t>jamais moins de 20 ms, seuil courant de perception d'un décalage</t>
         </is>
       </c>
     </row>
@@ -4450,27 +4485,27 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>± 120</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>ms</t>
+          <t>% de la ½ subdivision</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>fixe en phase 1</t>
+          <t>réglages</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -4480,7 +4515,7 @@
       </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
-          <t>deviendra réglable en phase 2</t>
+          <t>à 100 %, le graphe couvre exactement la plage qu'un écart peut atteindre</t>
         </is>
       </c>
     </row>
@@ -4782,7 +4817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5258,6 +5293,72 @@
         </is>
       </c>
     </row>
+    <row r="23" ht="45.75" customHeight="1">
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>Tolérance absolue ou relative à la subdivision</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>Une zone juste réglée en millisecondes vaut la même largeur quelle que soit la grille : ±50 ms représentent 5 % de l'intervalle sur une noire à 60 bpm, mais 43 % sur une double-croche à 128 bpm, où l'app validerait un placement qui s'entend comme maladroit.</t>
+        </is>
+      </c>
+      <c r="C23" s="20" t="inlineStr">
+        <is>
+          <t>Exprimée en pourcentage de la subdivision, avec plancher absolu à 20 ms — la même forme que le seuil de régularité (EX-082), pour la même raison : un pourcentage seul finirait par exiger mieux que ce qu'une main peut faire et qu'une oreille peut entendre. Un seul curseur, pas de bascule ms/% à maintenir.</t>
+        </is>
+      </c>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>Un « dans la zone » qui ne veut pas dire la même chose d'un tempo à l'autre, donc inutilisable pour se comparer d'une séance à la suivante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="45.75" customHeight="1">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>Moyenne glissante seule comme lecture instantanée</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>Première version du vu-mètre alimentée par la seule moyenne des 16 dernières notes. À l'essai, il restait au vert quoi qu'on joue : les écarts en avance annulent ceux en retard. Vérifié sur un enregistrement réel — des notes à ±51 ms, 6 sur 16 hors zone, et une moyenne qui ne sortait jamais de ±11 ms.</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>La moyenne mesure le biais, pas la précision. Le vu-mètre couvre désormais la fourchette moyenne ± dispersion, chaque côté s'allumant indépendamment, et le verdict gagne un état « irrégulier » pour le jeu dispersé mais centré.</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>Un indicateur qui félicite un jeu approximatif — le contraire exact de ce que l'application sert à faire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="45.75" customHeight="1">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>Vu-mètre à neuf barres graduées</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>Première forme retenue pour la lecture instantanée : neuf barres, chacune large de deux fois la tolérance. La largeur d'une tranche dépendait donc d'un réglage utilisateur. À l'essai, avec une tolérance généreuse (croches à 84 bpm, ~15 %), une barre valait 107 ms : toute une performance à ±103 ms tenait dans une seule barre de chaque côté, et six barres sur neuf restaient éteintes en permanence.</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="inlineStr">
+        <is>
+          <t>Réduit à trois voyants — triangle, barre, triangle. La direction et l'état irrégulier subsistent ; l'ampleur du décalage est portée par la valeur chiffrée et la ligne de statistiques, qui l'expriment mieux qu'un nombre de barres.</t>
+        </is>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>Une résolution affichée que la mesure ne remplit jamais : l'utilisateur croit l'indicateur figé alors qu'il fonctionne.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Track deliberate tempo changes in one beat instead of twenty
Smoothing the MIDI clock period absorbs jitter well but took ~10 beats to
reach a tempo just dialled in on the keyboard — and because the phase
correction is capped at 20 ms per beat, it could not catch up with a period
that far off: the click drifted up to 220 ms from the true beat and needed
21 beats to recover. The metronome was genuinely wrong for ten seconds after
every tempo change, not merely slow to display.

Weakening the smoothing would pay permanent jitter for a one-off gain, so
instead an interval more than 8% off the current estimate is taken as a
deliberate change and adopted outright. The threshold clears normal transport
jitter (~1%) and a dropped clock pulse (4.2%) by a wide margin.
</commit_message>
<xml_diff>
--- a/JustRhythm/cahier-des-charges-just-rhythm-natif.xlsx
+++ b/JustRhythm/cahier-des-charges-just-rhythm-natif.xlsx
@@ -815,7 +815,7 @@
     <row r="42" ht="82" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>v2.4 — Lecture instantanée sur la fourchette glissante. L'écart de la dernière note, trop instable pour qu'on s'y fie en jouant, cède la place à trois voyants façon accordeur, alimentés par la moyenne et la dispersion des 16 dernières notes (EX-066 / EX-089, cette dernière passant en phase 1) : les deux côtés s'allument séparément, ce qui distingue un décalage systématique d'un jeu irrégulier. Le tempo reçu du clavier est désormais adopté par l'application et conservé après l'arrêt, les commandes de tempo étant neutralisées tant que l'horloge pilote (EX-054).</t>
+          <t>v2.4 — Lecture instantanée sur la fourchette glissante. L'écart de la dernière note, trop instable pour qu'on s'y fie en jouant, cède la place à trois voyants façon accordeur, alimentés par la moyenne et la dispersion des 16 dernières notes (EX-066 / EX-089, cette dernière passant en phase 1) : les deux côtés s'allument séparément, ce qui distingue un décalage systématique d'un jeu irrégulier. Le tempo reçu du clavier est désormais adopté par l'application et conservé après l'arrêt, les commandes de tempo étant neutralisées tant que l'horloge pilote (EX-054). Un changement de tempo au clavier est désormais suivi en un temps au lieu d'une vingtaine.</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2844,7 @@
       </c>
       <c r="D50" s="33" t="inlineStr">
         <is>
-          <t>Suivi de l'horloge MIDI (24 impulsions par noire). Période lissée et phase corrigée par un décalage d'ancrage borné, sans rupture de grille. Le tempo reçu est affiché à la place du tempo réglé, qui ne fait plus foi, et il est adopté comme tempo de l'application : les réglages qui en dépendent le suivent, et la valeur survit à l'arrêt de la séance. Les commandes de tempo sont neutralisées tant que l'horloge pilote. S'active et se désactive avec EX-053 : un seul réglage « Démarrage synchronisé » commande les deux, il n'y a jamais de cas où l'un est utile sans l'autre.</t>
+          <t>Suivi de l'horloge MIDI (24 impulsions par noire). Période lissée et phase corrigée par un décalage d'ancrage borné, sans rupture de grille — sauf écart franc (plus de 8 %), reconnu comme un tempo changé au clavier et adopté d'un coup, sans quoi le clic mettrait une vingtaine de temps à revenir sur le temps. Le tempo reçu est affiché à la place du tempo réglé, qui ne fait plus foi, et il est adopté comme tempo de l'application : les réglages qui en dépendent le suivent, et la valeur survit à l'arrêt de la séance. Les commandes de tempo sont neutralisées tant que l'horloge pilote. S'active et se désactive avec EX-053 : un seul réglage « Démarrage synchronisé » commande les deux, il n'y a jamais de cas où l'un est utile sans l'autre.</t>
         </is>
       </c>
       <c r="E50" s="36" t="inlineStr">
@@ -4817,7 +4817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5359,6 +5359,28 @@
         </is>
       </c>
     </row>
+    <row r="26" ht="45.75" customHeight="1">
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>Lissage de l'horloge et réponse à un changement de tempo</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>Le lissage de la période (moyenne exponentielle à 0,2 par temps) absorbe bien la gigue, mais met une dizaine de temps à rejoindre un tempo changé sur le clavier. Pire : la correction de phase étant bornée à 20 ms par temps, elle ne rattrape pas une période fausse de 100 ms — en simulation, le clic s'écarte jusqu'à 220 ms du vrai temps et met 21 temps à revenir. Affaiblir le lissage paie de la gigue en permanence pour un gain ponctuel, et avait été essayé puis annulé plus tôt : l'échec d'alors venait en réalité de l'amplification par stepIndex, pas du lissage.</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>Lissage conservé tel quel, doublé d'une détection de changement franc : au-delà de 8 % d'écart avec l'estimation courante, l'intervalle est adopté sans lissage. Le seuil passe largement au-dessus de la gigue (de l'ordre du pour cent) et de la perte d'une impulsion d'horloge (4,2 %). Réponse en un temps, sans gigue ajoutée.</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>Un métronome qui reste faux une dizaine de secondes après chaque changement de tempo, et qu'on croit déréglé alors qu'il converge.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Prepare v2.4 for App Store submission
Version bumped to 2.4 (build 7), aligned with spec document rather than
incremental versioning. Build 1.0(2) corresponds to v2.1 state; this release
incorporates v2.2–v2.4 fixes: MIDI clock drift elimination, note counter
persistence, source fallback restoration, tuner-readout instant feedback,
and keyboard tempo adoption.

- Update MARKETING_VERSION to 2.4, CURRENT_PROJECT_VERSION to 7
- Add CHANGELOG.md documenting v2.0–v2.4 with decision traceability
- Replace preview screenshots (A.png, B.png, C.png) with current app state,
  resized to 1284×2778 (6.5" category)
- Remove stale video preview (C-conforme.mp4)
- Document v2.4 and simulator limitations in spec decision log

xcodebuild -scheme JustRhythm -sdk iphonesimulator build: SUCCESS

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/JustRhythm/cahier-des-charges-just-rhythm-natif.xlsx
+++ b/JustRhythm/cahier-des-charges-just-rhythm-natif.xlsx
@@ -4837,7 +4837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5445,6 +5445,50 @@
         </is>
       </c>
     </row>
+    <row r="29" ht="45.75" customHeight="1">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>Numérotation App Store alignée sur le cahier des charges</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>Le premier binaire soumis, 1.0 (2), a été archivé le 28/07/2026 : son numéro de build n'apparaît nulle part dans l'historique, qui passe de 1 à 3 le même jour. Il correspond donc à l'état v2.1 — antérieur à la correction de la dérive de synchro (v2.2), à la justesse rapportée à la subdivision (v2.3) et aux voyants de lecture instantanée (v2.4).</t>
+        </is>
+      </c>
+      <c r="C29" s="20" t="inlineStr">
+        <is>
+          <t>La publication suivante portera le numéro 2.4, aligné sur celui du cahier des charges plutôt que sur une suite 1.1. App Store Connect n'exige qu'une version strictement supérieure à la précédente, comparée composant par composant : 1.0 → 2.4 passe, et les numéros sautés ne déclenchent aucun contrôle. L'alignement permet à un utilisateur qui signale « je suis en 2.4 » de pointer directement une ligne du journal. Le numéro de build, lui, ne se remet jamais à 1 : il continue en 7.</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>Une version publiée qu'on ne sait plus rattacher à un état du cahier des charges, et un envoi refusé si le couple version + build repasse sur une valeur déjà reçue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="45.75" customHeight="1">
+      <c r="A30" s="22" t="inlineStr">
+        <is>
+          <t>Captures d'écran impossibles depuis le simulateur</t>
+        </is>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>Le simulateur iOS ne partage pas le CoreMIDI du Mac : une source MIDI virtuelle créée sur l'hôte reste invisible de l'application, même après relance pour forcer un nouveau balayage — « Clavier : aucun détecté ». Sans clavier, le graphe reste vide et les statistiques à zéro.</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="inlineStr">
+        <is>
+          <t>Les captures de la fiche App Store se prennent sur l'iPhone, clavier branché, en séance réelle. Le simulateur ne sert qu'à vérifier la mise en page. Les dimensions sont conformées ensuite par resize-screenshots.sh, catégorie 6,5 pouces (1284×2778).</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="inlineStr">
+        <is>
+          <t>Du temps passé à outiller une injection MIDI qui ne peut pas aboutir, ou une fiche App Store illustrée par une application qui paraît ne rien faire.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Scale the keyboard-feedback safety release to one bar
The forced release that catches a lost Note Off was a flat ten seconds, which
does not mean the same thing at 40 and at 200 bpm. It is now exactly one bar,
computed through the grid period, so it follows the keyboard's MIDI clock when
that clock is being followed.

One bar and not more: the choice is to keep the net tight, accepting that a
note held past a bar line has its echo cut short, rather than let a stray note
settle in. No clamping is needed — tempo is already bounded to 30-240 bpm and
beats per bar to 12, so the value stays between 0.5 s and 24 s.

Still v2.5: this refines the feedback behaviour introduced in a93b437, it does
not add to it. Requirements document, CHANGELOG and both user manuals updated;
the decision log records the trade-off as a deliberate choice.

xcodebuild -scheme JustRhythm -sdk iphonesimulator build: SUCCESS

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/JustRhythm/cahier-des-charges-just-rhythm-natif.xlsx
+++ b/JustRhythm/cahier-des-charges-just-rhythm-natif.xlsx
@@ -623,7 +623,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -645,7 +644,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="19.5" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
@@ -660,7 +658,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="19.5" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -689,7 +686,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="19.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -704,7 +700,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="19.5" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -719,7 +714,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="19.5" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
@@ -734,7 +728,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25" ht="19.5" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
@@ -749,7 +742,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28" ht="19.5" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
         <is>
@@ -764,7 +756,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31" ht="19.5" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
@@ -786,7 +777,6 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
     <row r="35" ht="19.5" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
@@ -801,7 +791,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38" ht="19.5" customHeight="1">
       <c r="A38" s="3" t="inlineStr">
         <is>
@@ -816,7 +805,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41" ht="19.5" customHeight="1">
       <c r="A41" s="3" t="inlineStr">
         <is>
@@ -873,7 +861,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
@@ -4182,7 +4169,7 @@
       </c>
       <c r="D84" s="33" t="inlineStr">
         <is>
-          <t>Une section « Retour clavier » dans les Réglages, avec un interrupteur « Renvoyer une note quand la frappe est juste », désactivé par défaut. Actif, il envoie un Note On vers l'instrument à chaque frappe tombée dans la zone « juste », et le Note Off correspondant au lever de la touche qui l'a déclenché : la note de retour dure exactement ce que dure le geste. Aucune note ne survit à son déclencheur — relâchement forcé au bout de 10 s si le Note Off se perd, extinction générale à l'arrêt, à la coupure du réglage et à la perte de la source.</t>
+          <t>Une section « Retour clavier » dans les Réglages, avec un interrupteur « Renvoyer une note quand la frappe est juste », désactivé par défaut. Actif, il envoie un Note On vers l'instrument à chaque frappe tombée dans la zone « juste », et le Note Off correspondant au lever de la touche qui l'a déclenché : la note de retour dure exactement ce que dure le geste. Aucune note ne survit à son déclencheur — relâchement forcé au bout d'une mesure si le Note Off se perd, et extinction générale à l'arrêt, à la coupure du réglage et à la perte de la source.</t>
         </is>
       </c>
       <c r="E84" s="36" t="inlineStr">
@@ -5560,7 +5547,7 @@
       </c>
       <c r="C31" s="20" t="inlineStr">
         <is>
-          <t>La durée n'est plus calculée du tout. Note On à l'appui, Note Off au lever de la touche qui l'a déclenché : le retour dure exactement ce que dure le geste, quel que soit le tempo, la subdivision ou l'écriture. L'objection initiale — « on ne connaît pas la durée à l'attaque » — tombe dès qu'on cesse de vouloir la connaître : il suffit de relayer le relâchement quand il arrive. La correspondance touche jouée → note renvoyée est mémorisée, et non recalculée, pour survivre à un changement de mode en cours de note ; les notes envoyées sont décomptées, pour qu'un lever n'éteigne pas le retour d'une autre touche qui porte le même numéro.</t>
+          <t>La durée n'est plus calculée du tout. Note On à l'appui, Note Off au lever de la touche qui l'a déclenché : le retour dure exactement ce que dure le geste, quel que soit le tempo, la subdivision ou l'écriture. L'objection initiale — « on ne connaît pas la durée à l'attaque » — tombe dès qu'on cesse de vouloir la connaître : il suffit de relayer le relâchement quand il arrive. La correspondance touche jouée → note renvoyée est mémorisée, et non recalculée, pour survivre à un changement de mode en cours de note ; les notes envoyées sont décomptées, pour qu'un lever n'éteigne pas le retour d'une autre touche qui porte le même numéro. Le filet contre un Note Off perdu vaut une mesure — rapporté à la grille comme le reste, là où dix secondes fixes ne voulaient pas dire la même chose à 40 et à 200 bpm. Une mesure et non deux : le choix est de garder le filet serré, en acceptant qu'une note tenue par-dessus une barre de mesure soit écourtée, plutôt que de laisser une note fantôme s'installer. Aucune borne n'est nécessaire, le tempo étant déjà limité à 30-240 bpm et les temps par mesure à 12 : la valeur va de 0,5 s à 24 s.</t>
         </is>
       </c>
       <c r="D31" s="20" t="inlineStr">

</xml_diff>